<commit_message>
adding the feature for multiple paper types
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,6 +432,11 @@
           <t>Password</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Paper Type</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -446,7 +451,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>OVVQEWX2</t>
+          <t>9KU7bkdF</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -463,7 +473,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>9niXrSj0</t>
+          <t>ftNbcELK</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -480,7 +495,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ThTpCHw9</t>
+          <t>yl2iaN7S</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -497,7 +517,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>oWiEYt5V</t>
+          <t>6YsWeWDx</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -514,7 +539,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>g1pHN9UO</t>
+          <t>AE5Vf5CJ</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -531,7 +561,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>94qwcReE</t>
+          <t>jP7fi32d</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -548,7 +583,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ABXvCm4y</t>
+          <t>RItEKdUH</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -565,7 +605,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>wzQ6flh5</t>
+          <t>vcTmXOQ0</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -582,7 +627,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Dq08qlKB</t>
+          <t>LgE6Afoa</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -599,7 +649,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>oQQbahNb</t>
+          <t>aVJiHhFA</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -616,7 +671,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>qQ1ioq0r</t>
+          <t>qAP17DEK</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -633,7 +693,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>qSs15eyk</t>
+          <t>njjo7JLn</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -650,7 +715,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>HdYyK5St</t>
+          <t>I2EgIuYq</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -667,7 +737,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>xMEY0Rx5</t>
+          <t>sDmf3GDc</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -684,7 +759,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>qnzFdDrF</t>
+          <t>pLQhHsJH</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -701,7 +781,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>WFHbSMFL</t>
+          <t>nSYSqDe4</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -718,7 +803,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>58TOtEuD</t>
+          <t>rOkeqmG6</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -735,7 +825,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>xvWBVCqW</t>
+          <t>NitsNXs6</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -752,7 +847,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>7YEBn6V5</t>
+          <t>AMhQbGKI</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -769,7 +869,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>3IvlRxrj</t>
+          <t>5Tey3906</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -786,7 +891,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>dDTOENha</t>
+          <t>oHVvSzTI</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -803,7 +913,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>xvxbY5IV</t>
+          <t>BLCOFhDa</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -820,7 +935,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>qqLEUTXY</t>
+          <t>abxsl9S1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -837,7 +957,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>5VhURI7s</t>
+          <t>JbZpOStH</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -854,7 +979,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>hS3bYcha</t>
+          <t>SoYsLQlX</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -871,7 +1001,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>vHugA1r8</t>
+          <t>8cMzu0Oe</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -888,7 +1023,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>zPvL2Mdo</t>
+          <t>yNt4Ctev</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -905,7 +1045,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>6T5NJxNr</t>
+          <t>oHHRkFC8</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -922,7 +1067,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>cVRHISh2</t>
+          <t>8rGmwd8N</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -939,7 +1089,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>dXcuOVCN</t>
+          <t>jGgmT5aR</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -956,7 +1111,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Gl71rUzQ</t>
+          <t>0Ky13CME</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -973,7 +1133,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>D4m62ccD</t>
+          <t>Yy93mlMs</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -990,7 +1155,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>dipj4csz</t>
+          <t>SiWKKAg6</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1177,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>fRsvJ2L1</t>
+          <t>Zv19VN7g</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1199,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>HVT2KuiQ</t>
+          <t>wplt9wwh</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1221,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>UuGoyN1G</t>
+          <t>M7TNwnGZ</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
     </row>
@@ -1054,7 +1239,12 @@
       <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
-          <t>rlSVZ01v</t>
+          <t>6Ef4hQmZ</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
adding two games for the students
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,7 +451,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Q4rZdaqp</t>
+          <t>n9W80bJq</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -473,7 +473,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Rlw71Hrs</t>
+          <t>0S0fEnJ3</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -495,7 +495,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>wKt4RGmT</t>
+          <t>CpOZdKWJ</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -517,10 +517,54 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>BzXJaXsV</t>
+          <t>2SvnK7o9</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>20P-0005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Test 5</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>lOHsg2aC</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>20P-0006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Test 6</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>FO6mW9Qb</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
         <is>
           <t>A</t>
         </is>

</xml_diff>

<commit_message>
[200~Switch server to threaded request handling, add thread-safe session/data access with Excel caching, and gracefully handle broken client connections to prevent noisy 500 traces under load. Also refresh README with complete admin/student runbook, scaling notes, LAN/firewall checks, and troubleshooting guidance.
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -413,158 +413,1306 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>S#</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Roll No.</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Student Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Password</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Paper Type</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>20P-0001</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Test 1</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>n9W80bJq</t>
-        </is>
-      </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>ufxOZeRe</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>20P-0002</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Test 2</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>0S0fEnJ3</t>
-        </is>
-      </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>srOQyCvw</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>20P-0003</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Test 3 </t>
-        </is>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CpOZdKWJ</t>
+          <t>Test 3</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
+          <t>ZhToC6Q8</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>20P-0004</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Test 4</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2SvnK7o9</t>
-        </is>
-      </c>
       <c r="D5" t="inlineStr">
         <is>
+          <t>8YsNHhtg</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>20P-0005</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Test 5</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>lOHsg2aC</t>
-        </is>
-      </c>
       <c r="D6" t="inlineStr">
         <is>
+          <t>hHCxRx5C</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>A</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>20P-0006</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Test 6</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>FO6mW9Qb</t>
-        </is>
-      </c>
       <c r="D7" t="inlineStr">
+        <is>
+          <t>L8qqPxQD</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>20P-0007</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Test 7</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>F3wXbiL0</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>20P-0008</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Test 8</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0L7Qmn8S</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>20P-0009</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Test 9</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>eUaAzsdI</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>20P-0010</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Test 10</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>7lsg3Lb5</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>20P-0011</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Test 11</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Z2P4YTzR</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>20P-0012</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Test 12</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>vZ3jyGEZ</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>20P-0013</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Test 13</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>UFdoOxk4</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>20P-0014</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Test 14</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>n2LghhXl</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>20P-0015</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Test 15</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>vUARHbJO</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>20P-0016</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Test 16</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>JQRt72Rl</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>20P-0017</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Test 17</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>sxF9YH7v</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>20P-0018</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Test 18</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Av4ZqR2Z</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>20P-0019</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Test 19</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>sAa3kk0s</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>20P-0020</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Test 20</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>kw9WeDPn</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>20P-0021</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Test 21</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>GlPVNJTu</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>20P-0022</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Test 22</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>cXoOvHZU</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>20P-0023</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Test 23</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>NPvsiucp</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>20P-0024</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Test 24</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ENzlpTb9</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>20P-0025</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Test 25</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>jSt37Xgt</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>20P-0026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Test 26</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>WZbsLqTM</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>20P-0027</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Test 27</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>iIk3HSki</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>20P-0028</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Test 28</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>kefDnn6G</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>20P-0029</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Test 29</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>k1Jv0twj</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>20P-0030</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Test 30</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>WLkBxyYU</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>20P-0031</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Test 31</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>73Mqa6gU</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>20P-0032</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Test 32</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>JBPVCql6</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>20P-0033</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Test 33</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>uWwP2fb2</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>20P-0034</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Test 34</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>HVOl3gD4</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>20P-0035</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Test 35</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>ugIexFEN</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>20P-0036</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Test 36</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>I6FdLAsN</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>20P-0037</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Test 37</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>h8TbSbbd</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>20P-0038</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Test 38</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>hviCfJNF</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>20P-0039</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Test 39</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>xdw5CZ3Z</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>20P-0040</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Test 40</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>vUAcPzag</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>20P-0041</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Test 41</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>ArUt1dP5</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>20P-0042</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Test 42</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>qYQsH1U1</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>20P-0043</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Test 43</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>YCHxsYnF</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>20P-0044</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Test 44</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>XO0ovgQW</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>20P-0045</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Test 45</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>lppCKWn9</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>20P-0046</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Test 46</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>pBIiM0oV</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>20P-0047</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Test 47</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>ic2SCkck</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>20P-0048</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Test 48</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>c5r5vPTR</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>20P-0049</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Test 49</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ZCJXp9NZ</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>20P-0050</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Test 50</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>UBJoTb5V</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>20P-0051</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Test 51</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>JnU61WSr</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>A</t>
         </is>

</xml_diff>

<commit_message>
added timer, file size, file type, hyperlink to the directory, some panel updates
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,17 +449,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>20P-0001</t>
+          <t>20P-0070</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Test 1</t>
+          <t>Qasim Ali</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>ufxOZeRe</t>
+          <t>iT1lilhb</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -474,17 +474,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>20P-0002</t>
+          <t>22P-9065</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Test 2</t>
+          <t>Hamza Tahir</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>srOQyCvw</t>
+          <t>rfmLDVlp</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -499,17 +499,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>20P-0003</t>
+          <t>22P-9411</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Test 3</t>
+          <t>Muhammad Farooq Farooqi</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ZhToC6Q8</t>
+          <t>vE8q8LIk</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -524,17 +524,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>20P-0004</t>
+          <t>23P-3008</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Test 4</t>
+          <t>Talha Khan</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8YsNHhtg</t>
+          <t>yiXMgCNe</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -549,17 +549,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>20P-0005</t>
+          <t>23P-3023</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Test 5</t>
+          <t>Wajahat Taj</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>hHCxRx5C</t>
+          <t>x4V51EE1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -574,17 +574,17 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>20P-0006</t>
+          <t>24P-0003</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Test 6</t>
+          <t>Muhammad Hamza</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>L8qqPxQD</t>
+          <t>3PoR7imS</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -599,17 +599,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>20P-0007</t>
+          <t>24P-0503</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Test 7</t>
+          <t>Syed Muhammad Iqan Hashmi</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>F3wXbiL0</t>
+          <t>Kc6F5mM8</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -624,17 +624,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>20P-0008</t>
+          <t>24P-0520</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Test 8</t>
+          <t>Arbab Arsalan Khalil</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0L7Qmn8S</t>
+          <t>6CdFNegC</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -649,17 +649,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>20P-0009</t>
+          <t>24P-0527</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Test 9</t>
+          <t>Manahil Fatima</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>eUaAzsdI</t>
+          <t>gCskUWpH</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -674,17 +674,17 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>20P-0010</t>
+          <t>24P-0528</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Test 10</t>
+          <t>Muhammad Rayan</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>7lsg3Lb5</t>
+          <t>QjHUYMvM</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -699,17 +699,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>20P-0011</t>
+          <t>24P-0553</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Test 11</t>
+          <t>Waleed Orakzai</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Z2P4YTzR</t>
+          <t>tNW6ZmId</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -724,17 +724,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>20P-0012</t>
+          <t>24P-0557</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Test 12</t>
+          <t>Hafiz Muhammad Umer Abdullah</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>vZ3jyGEZ</t>
+          <t>xRXw19gA</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -749,17 +749,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>20P-0013</t>
+          <t>24P-0561</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Test 13</t>
+          <t>Taha Yasin</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>UFdoOxk4</t>
+          <t>E5tNK1VT</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -774,17 +774,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>20P-0014</t>
+          <t>24P-0564</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Test 14</t>
+          <t>Saad Ali</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>n2LghhXl</t>
+          <t>rMxcC051</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -799,17 +799,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>20P-0015</t>
+          <t>24P-0568</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Test 15</t>
+          <t>Momin Tahoor</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>vUARHbJO</t>
+          <t>JbqPiLHF</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -824,17 +824,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>20P-0016</t>
+          <t>24P-0569</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Test 16</t>
+          <t>Muhammad Muneeb Khan</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>JQRt72Rl</t>
+          <t>yastBhfP</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>20P-0017</t>
+          <t>24P-0572</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Test 17</t>
+          <t>Sudais Khan</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>sxF9YH7v</t>
+          <t>lDMbYKvg</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -874,17 +874,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>20P-0018</t>
+          <t>24P-0573</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Test 18</t>
+          <t>Shayan Ali</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Av4ZqR2Z</t>
+          <t>kYBko5BM</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -899,17 +899,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>20P-0019</t>
+          <t>24P-0576</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Test 19</t>
+          <t>Asawir Binte Asif</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>sAa3kk0s</t>
+          <t>DuU6syyZ</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -924,17 +924,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>20P-0020</t>
+          <t>24P-0603</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Test 20</t>
+          <t>Muhammad Israr</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>kw9WeDPn</t>
+          <t>4VsIwIqK</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -949,17 +949,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>20P-0021</t>
+          <t>24P-0615</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Test 21</t>
+          <t>Rahim Alam</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>GlPVNJTu</t>
+          <t>k6Oxgx1Z</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -974,17 +974,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>20P-0022</t>
+          <t>24P-0623</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Test 22</t>
+          <t>Hizb Ullah</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>cXoOvHZU</t>
+          <t>2124PFBb</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -999,17 +999,17 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>20P-0023</t>
+          <t>24P-0634</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Test 23</t>
+          <t>Syed Muhammad Hussain Hammad</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>NPvsiucp</t>
+          <t>uPlEOIxu</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1024,17 +1024,17 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>20P-0024</t>
+          <t>24P-0641</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Test 24</t>
+          <t>Muhammad Afnan Khan</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>ENzlpTb9</t>
+          <t>MFfXPoXO</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1049,17 +1049,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>20P-0025</t>
+          <t>24P-0652</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Test 25</t>
+          <t>Anas Malik</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>jSt37Xgt</t>
+          <t>Lkt2rPbc</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1074,17 +1074,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>20P-0026</t>
+          <t>24P-0660</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Test 26</t>
+          <t>Zia Ullah</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>WZbsLqTM</t>
+          <t>VaIO5mD3</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1099,17 +1099,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>20P-0027</t>
+          <t>24P-0661</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Test 27</t>
+          <t>Ahmed Ali Hassan</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>iIk3HSki</t>
+          <t>KXQgCebv</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1124,17 +1124,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>20P-0028</t>
+          <t>24P-0671</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Test 28</t>
+          <t>Muhammad Hamza Shahzad</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>kefDnn6G</t>
+          <t>csT7n537</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1149,17 +1149,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>20P-0029</t>
+          <t>24P-0672</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Test 29</t>
+          <t>Syed Muhammad Qasim</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>k1Jv0twj</t>
+          <t>tRBTIMzT</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1174,17 +1174,17 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>20P-0030</t>
+          <t>24P-0686</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Test 30</t>
+          <t>Talha Arshad</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>WLkBxyYU</t>
+          <t>B9vd79Fe</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -1199,17 +1199,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>20P-0031</t>
+          <t>24P-0715</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Test 31</t>
+          <t>Sudais Khan Burki</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>73Mqa6gU</t>
+          <t>HoHJF1hf</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1224,17 +1224,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>20P-0032</t>
+          <t>24P-0732</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Test 32</t>
+          <t>Muhammad Sohaib Bukhari</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>JBPVCql6</t>
+          <t>mTNm2Uwb</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1249,17 +1249,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>20P-0033</t>
+          <t>24P-0733</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Test 33</t>
+          <t>Muhammad Bin Nawaz Ul Haq</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>uWwP2fb2</t>
+          <t>LQP5AuFJ</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1274,17 +1274,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>20P-0034</t>
+          <t>24P-0742</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Test 34</t>
+          <t>Mueez Khalid</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>HVOl3gD4</t>
+          <t>K8dBr2sz</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1299,17 +1299,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>20P-0035</t>
+          <t>24P-3120</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Test 35</t>
+          <t>Junaid Nawab</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>ugIexFEN</t>
+          <t>goaEuG4X</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1324,17 +1324,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>20P-0036</t>
+          <t>24P-3131</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Test 36</t>
+          <t>Yasir Hameed</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>I6FdLAsN</t>
+          <t>jB4AjQT2</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1349,17 +1349,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>20P-0037</t>
+          <t>23P-3063</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Test 37</t>
+          <t>Muhammad Anas Imran</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>h8TbSbbd</t>
+          <t>369R56SV</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1374,17 +1374,17 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>20P-0038</t>
+          <t>24K-0925</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Test 38</t>
+          <t>Ahmed Hassan</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>hviCfJNF</t>
+          <t>NCBNNEJc</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1399,17 +1399,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>20P-0039</t>
+          <t>24P-0500</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Test 39</t>
+          <t>Mehr Ali</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>xdw5CZ3Z</t>
+          <t>0zQhhA3g</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1424,17 +1424,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>20P-0040</t>
+          <t>24P-0509</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Test 40</t>
+          <t>Syed Saifullah Shah</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>vUAcPzag</t>
+          <t>CHcT7Kf6</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1449,17 +1449,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>20P-0041</t>
+          <t>24P-0518</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Test 41</t>
+          <t>Abdul Rehman</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>ArUt1dP5</t>
+          <t>P48ySkdE</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1474,17 +1474,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>20P-0042</t>
+          <t>24P-0524</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Test 42</t>
+          <t>Muhammad Muddasir</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>qYQsH1U1</t>
+          <t>3kQ473Bp</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1499,17 +1499,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>20P-0043</t>
+          <t>24P-0530</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Test 43</t>
+          <t>Muhammad Bilal</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>YCHxsYnF</t>
+          <t>Y110Ggz6</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1524,17 +1524,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>20P-0044</t>
+          <t>24P-0548</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Test 44</t>
+          <t>Talha Khan</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>XO0ovgQW</t>
+          <t>dZTKL6sc</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1549,17 +1549,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>20P-0045</t>
+          <t>24P-0562</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Test 45</t>
+          <t>Muhammad Safwan Ghani</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>lppCKWn9</t>
+          <t>niqvZrZa</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1574,17 +1574,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>20P-0046</t>
+          <t>24P-0570</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Test 46</t>
+          <t>Qazi Abdur Rahman</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>pBIiM0oV</t>
+          <t>Doz2iXv6</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -1599,17 +1599,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>20P-0047</t>
+          <t>24P-0575</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Test 47</t>
+          <t>Ali Hamza Saifi</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>ic2SCkck</t>
+          <t>03tIFdrP</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -1624,17 +1624,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>20P-0048</t>
+          <t>24P-0580</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Test 48</t>
+          <t>Sultan Taimoor Wadood Mufti</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>c5r5vPTR</t>
+          <t>htUauN1L</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -1649,17 +1649,17 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>20P-0049</t>
+          <t>24P-0581</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Test 49</t>
+          <t>Muhammad Zaid Bin Arif</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>ZCJXp9NZ</t>
+          <t>Asb60rji</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -1674,17 +1674,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>20P-0050</t>
+          <t>24P-0584</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Test 50</t>
+          <t>Syed Zuhair Asim</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>UBJoTb5V</t>
+          <t>Qzw0FvdT</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -1699,20 +1699,2695 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>20P-0051</t>
+          <t>24P-0594</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Test 51</t>
+          <t>Haziqa Eiman</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>JnU61WSr</t>
+          <t>lK3TtdRN</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>24P-0595</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Ayesha Anees</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>PPVi06uv</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>24P-0597</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Muhammad Talha</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>5ljnY09F</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>24P-0599</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Sherbano Naveed</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>hCYXSbyM</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>24P-0600</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Muhammad Ibrahim Fakhir</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>EHpeiAT6</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>24P-0604</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Sohrab</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>X5c9scWw</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>24P-0605</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Imdad Ali</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>GOkWYwnD</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>24P-0607</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Ali Irtaza Abbas Siddiqui</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>SKeO8zyo</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>24P-0608</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Abu Waqas</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>2j9ew5ya</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>24P-0609</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Haleema Sadia</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>hSqjegzm</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>24P-0616</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Behzad Tariq</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>n1FxM5rF</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>24P-0618</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Syed Ali Hussain Shah</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>ZgoN6sON</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>24P-0619</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Muhammad Musawar Ali Shah</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>YAw0iVzN</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>24P-0627</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Abdul Aziz</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Q02v6c1Z</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>24P-0646</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Muhammad Talha Shahid</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>y2ojFpRF</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>24P-0655</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Abdul Aziz</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>WHuhJAQu</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>24P-0656</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Muhammad Anwar</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>9cpKpdSy</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>24P-0665</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Muhammad Usman</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>p2IykYU4</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>24P-0668</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Yahya Bin Zia</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>dRnTqavA</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>24P-0674</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Fatima Waseem</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>UZhjUygX</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>24P-0676</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Fida Hussain</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>M6BIm0Y0</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>24P-0677</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Muhammad Azan</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>ECSF0Gho</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>24P-0698</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Syed Usman Ali Shah</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>mLAPdtDH</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>24P-0704</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Najaf Akash</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>StXxnaF6</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>24P-0711</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Aftab Ahmad</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>3fq27VFJ</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>24P-0723</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Muhammad Ali</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>q4z5yMru</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>24P-0743</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Wasi Kamal</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>1ntyQjlM</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>22P-9066</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Saad Ahmed</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Thst4EaH</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>22P-9228</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Talha Zia</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>crHOBgSD</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>23P-0651</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Eass Muhammad Naveed</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>RQoMF8Dj</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>24F-0722</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Abdullah Khan</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>9eC0ykRS</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>24P-0510</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Abdul Mueez</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>xEntqHrF</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>24P-0512</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Manaal Amir</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>b11awWn9</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>24P-0516</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Muhammad Sheharyar</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>aWXuw3bI</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>24P-0517</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Muhammad Abdal Khan</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>d5ilrd3F</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>24P-0523</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Abdul Azeem Javaid</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>KgdjgPHY</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>24P-0529</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Hisam Mehboob</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>obJFDLGs</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>24P-0537</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Syed Ammad Hussain Shah</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>gAhPljcw</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>24P-0542</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Muhammad Irshad</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>RjQWNT3s</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>24P-0549</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Sirajudin</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>5nlrXhxD</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>24P-0554</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Malik Muhammad Sanaullah</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>NnlH914x</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>24P-0556</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Marwa Mushtaq</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>jkE00MY1</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>24P-0571</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Muhammad Shoaib Shahid</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>UhWViPMj</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>24P-0586</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Mohammad Hashir</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>ZROEeVVD</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>24P-0587</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Hamza Rana</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>PGVf92NZ</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>24P-0590</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Sardar Umair Nawaz Khan</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>aLOP7zci</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>24P-0592</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Sheikh Saif Ali</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>rDWjPYRi</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>24P-0598</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Ahmad Mughal</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>FtmhSyur</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>24P-0610</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Arslan Tariq</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>QZiIpbuZ</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>24P-0613</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Ayaz Ali</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>WYmtnNiP</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>24P-0617</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Maimoona Naeem</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>SXjRBjZz</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>24P-0635</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Munesh Kumar</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>2Qw3ZfbQ</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>24P-0648</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Muhammad Ibrahim Khan Khattak</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>w9abapUn</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>24P-0659</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Muhammad Abdul Rafeh</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>TT1d6H9t</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>24P-0669</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Saad Ahmed Ijaz</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>R6hpWn70</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>24P-0683</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Zarish Imran</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>2yfku3RR</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>24P-0684</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Mirza Muaz Baig</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>RDcjdDTp</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>24P-0688</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Ahmad Abdullah</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>vfx2Zqvv</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>24P-0692</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Tanveer Ul Haq</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>yEaly1wz</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>24P-0694</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Yasir Ali</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>BMYz30YU</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>24P-0697</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Muhammad Usman</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>dnAmd6DI</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>24P-0701</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Muhammad Farhan</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>KIM5hieS</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>24P-0736</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Arif Ali</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>UT7riauG</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>24P-0740</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Muhammad Ahmed Asim</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>L6wINYBU</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>24P-0749</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Muhammad Bilal</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>mU3DHGgR</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>24P-0751</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Gohar Abbas</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>q5sE0HDc</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>24P-0759</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Abubakar Liaqat</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>FjDjlYjf</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>22P-9359</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Muhammad Aqsam Qureshi</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>K0W9yZCj</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>23P-0016</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Muhammad Sayil Raza</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>y4FPS1CX</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>24K-0853</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Hafiz Muhammad Fahad Ullah Khan</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>g1ZnySAu</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>24P-0048</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Kabeer Shoaib</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>oF0CSArL</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>24P-0501</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Muhammad Haseeb</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>2WMk6VPn</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>24P-0502</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Muhammad Rauf</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>UAY5wKpF</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>24P-0504</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Alishba Jawad</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>ncbhJoai</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>24P-0505</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Ayaan Jawad</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>rDKFOzRl</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>24P-0506</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Muhammad Shah Mir Khan</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>GycMj5nH</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>24P-0507</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Muhammad Uzair Shoaib</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>URNn2BZb</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>24P-0515</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Yasir Sultan</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>UcfcTbXA</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>24P-0522</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Ramsha Khalid</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>EHxVq0RC</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>24P-0525</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Haris Haider</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>Oa6xUs5A</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>24P-0534</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Muhammad Zaid</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>cG4rKczq</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>24P-0535</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Muhammad Ayyan</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>o9clMNqn</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>24P-0539</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Ahmad Moosa Sadiq</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>d8upYwga</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>24P-0540</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Muhammad Atif Khan</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>O3WdGJd3</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>24P-0545</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Muhammad Abbas</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>XYuLBB04</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>24P-0546</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Muhammad Azwar Khan</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>uUG2umEw</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>24P-0579</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Tayyaba Asif</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>s7fyze9c</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>24P-0593</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Muhammad Zaheeb</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>7Ngw5Oy6</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>24P-0596</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Muhammad Mohsin</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>K7GX1Zk8</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>24P-0601</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Abdul Rehman Mohammad Anwar</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>kGjyVwyz</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>24P-0606</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Muqeet Mahmood</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>pM3u01ck</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>24P-0621</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Munawar Ali</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>uFATlsvk</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>24P-0622</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Abdullah Mangrio</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>4UF5G1Gn</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>24P-0624</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Ibbad Ur Rehman</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>AtgIOjkr</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>24P-0638</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Muhammad Haris</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>zuY2Xoep</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>24P-0663</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Ayesha Zulfiqar</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>g5G1NWBv</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>24P-0680</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Muhammad Musif</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>GUN2SAD9</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>24P-0693</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Abbas Ahmed</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>O4RABIH2</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>24P-0703</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Abdul Basit</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>lCCNeuw0</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>24P-0706</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Aazan Noor Khuwaja</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>KhIDFPvC</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>24P-0722</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Muhammad  Rizwan Akbar</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>SAHgehuJ</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>24P-0724</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Abdul Rehman</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>U9VAmJzG</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>24P-0735</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Muhammad Abdullah Khan</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>hFLEkvvm</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>24P-0738</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Muhammad Bilal</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>96q0EaJU</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>24P-0741</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Ahmad Bilal Khan</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>AmyHhXQJ</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>24P-0745</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Sajid Islam</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>VEsDvx8t</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>24P-0748</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>Arham Ali</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>PrZryCCI</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>24P-0750</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Ayan Shibli</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>yXz1lRJ0</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
         <is>
           <t>A</t>
         </is>

</xml_diff>